<commit_message>
change data acknowledgement sheet name to statements
</commit_message>
<xml_diff>
--- a/eva_sub_cli/etc/EVA_Submission_Example.xlsx
+++ b/eva_sub_cli/etc/EVA_Submission_Example.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nkumar2/PycharmProjects/eva-sub-cli/eva_sub_cli/etc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59013E65-F413-9F4D-B203-F4C236F05526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25DCC83A-6AF8-EA4D-B6F6-8B419B37A2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16500" yWindow="-28200" windowWidth="51200" windowHeight="28200" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="16500" yWindow="-28200" windowWidth="51200" windowHeight="28200" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PLEASE READ FIRST" sheetId="1" r:id="rId1"/>
     <sheet name="Submitter Details" sheetId="2" r:id="rId2"/>
-    <sheet name="Data Acknowledgement" sheetId="12" r:id="rId3"/>
+    <sheet name="Statements" sheetId="12" r:id="rId3"/>
     <sheet name="Project HELP" sheetId="3" r:id="rId4"/>
     <sheet name="Project" sheetId="4" r:id="rId5"/>
     <sheet name="Analysis HELP" sheetId="5" r:id="rId6"/>
@@ -2382,16 +2382,48 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2399,17 +2431,11 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2432,32 +2458,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2745,8 +2745,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1025" s="5" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="72"/>
-      <c r="B1" s="66"/>
+      <c r="A1" s="70"/>
+      <c r="B1" s="71"/>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
@@ -2755,10 +2755,10 @@
       <c r="H1" s="4"/>
     </row>
     <row r="2" spans="1:1025" s="5" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="66"/>
+      <c r="B2" s="71"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -2767,10 +2767,10 @@
       <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:1025" s="5" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="75" t="s">
+      <c r="A3" s="74" t="s">
         <v>597</v>
       </c>
-      <c r="B3" s="66"/>
+      <c r="B3" s="71"/>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -2779,10 +2779,10 @@
       <c r="H3" s="7"/>
     </row>
     <row r="4" spans="1:1025" s="5" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="66"/>
+      <c r="B4" s="71"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -2791,10 +2791,10 @@
       <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:1025" s="5" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="73" t="s">
+      <c r="A5" s="80" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="66"/>
+      <c r="B5" s="71"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -3844,8 +3844,8 @@
       <c r="AMK7" s="5"/>
     </row>
     <row r="8" spans="1:1025" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="72"/>
-      <c r="B8" s="68"/>
+      <c r="A8" s="70"/>
+      <c r="B8" s="73"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -4871,10 +4871,10 @@
       <c r="AMK8" s="5"/>
     </row>
     <row r="9" spans="1:1025" ht="19" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="74" t="s">
+      <c r="A9" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="68"/>
+      <c r="B9" s="73"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
@@ -5900,8 +5900,8 @@
       <c r="AMK9" s="5"/>
     </row>
     <row r="10" spans="1:1025" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="72"/>
-      <c r="B10" s="68"/>
+      <c r="A10" s="70"/>
+      <c r="B10" s="73"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
@@ -6927,10 +6927,10 @@
       <c r="AMK10" s="5"/>
     </row>
     <row r="11" spans="1:1025" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="70" t="s">
+      <c r="A11" s="78" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="71"/>
+      <c r="B11" s="79"/>
     </row>
     <row r="12" spans="1:1025" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
@@ -6953,7 +6953,7 @@
       <c r="A14" s="16" t="s">
         <v>592</v>
       </c>
-      <c r="B14" s="87" t="s">
+      <c r="B14" s="65" t="s">
         <v>593</v>
       </c>
     </row>
@@ -6990,28 +6990,28 @@
       </c>
     </row>
     <row r="20" spans="1:1025" s="5" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="67" t="s">
+      <c r="A20" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="66"/>
+      <c r="B20" s="71"/>
     </row>
     <row r="21" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="67" t="s">
+      <c r="A21" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="68"/>
+      <c r="B21" s="73"/>
     </row>
     <row r="22" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="67" t="s">
+      <c r="A22" s="75" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="68"/>
+      <c r="B22" s="73"/>
     </row>
     <row r="23" spans="1:1025" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="67" t="s">
+      <c r="A23" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="68"/>
+      <c r="B23" s="73"/>
     </row>
     <row r="24" spans="1:1025" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="19"/>
@@ -9914,24 +9914,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="57" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="81" t="s">
         <v>592</v>
       </c>
-      <c r="B1" s="88"/>
-    </row>
-    <row r="2" spans="1:2" s="90" customFormat="1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A2" s="89" t="s">
+      <c r="B1" s="81"/>
+    </row>
+    <row r="2" spans="1:2" s="67" customFormat="1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="66" t="s">
         <v>594</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="66" t="s">
         <v>595</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="66" x14ac:dyDescent="0.2">
-      <c r="A3" s="91" t="b">
+      <c r="A3" s="68" t="b">
         <v>1</v>
       </c>
-      <c r="B3" s="92" t="s">
+      <c r="B3" s="69" t="s">
         <v>596</v>
       </c>
     </row>
@@ -10111,7 +10111,7 @@
       <c r="A1" s="30" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="78" t="s">
+      <c r="B1" s="84" t="s">
         <v>72</v>
       </c>
       <c r="C1" s="30" t="s">
@@ -10124,27 +10124,27 @@
     </row>
     <row r="2" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="20"/>
-      <c r="B2" s="79"/>
-      <c r="C2" s="76" t="s">
+      <c r="B2" s="85"/>
+      <c r="C2" s="82" t="s">
         <v>74</v>
       </c>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="77"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="83"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="73"/>
     </row>
     <row r="3" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="80"/>
+      <c r="B3" s="86"/>
       <c r="C3" s="20" t="s">
         <v>48</v>
       </c>
@@ -11029,15 +11029,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A1" s="85" t="s">
+      <c r="A1" s="91" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="78"/>
+      <c r="B1" s="92"/>
+      <c r="C1" s="84"/>
       <c r="D1" s="42" t="s">
         <v>218</v>
       </c>
-      <c r="E1" s="78" t="s">
+      <c r="E1" s="84" t="s">
         <v>72</v>
       </c>
       <c r="F1" s="42" t="s">
@@ -11087,63 +11087,63 @@
     <row r="2" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A2" s="48"/>
       <c r="B2" s="49"/>
-      <c r="C2" s="79"/>
+      <c r="C2" s="85"/>
       <c r="D2" s="50"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="81" t="s">
+      <c r="E2" s="85"/>
+      <c r="F2" s="87" t="s">
         <v>127</v>
       </c>
-      <c r="G2" s="82"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="82"/>
-      <c r="J2" s="82"/>
-      <c r="K2" s="83"/>
-      <c r="L2" s="84" t="s">
+      <c r="G2" s="88"/>
+      <c r="H2" s="88"/>
+      <c r="I2" s="88"/>
+      <c r="J2" s="88"/>
+      <c r="K2" s="89"/>
+      <c r="L2" s="90" t="s">
         <v>139</v>
       </c>
-      <c r="M2" s="82"/>
-      <c r="N2" s="83"/>
-      <c r="O2" s="84" t="s">
+      <c r="M2" s="88"/>
+      <c r="N2" s="89"/>
+      <c r="O2" s="90" t="s">
         <v>145</v>
       </c>
-      <c r="P2" s="82"/>
-      <c r="Q2" s="83"/>
-      <c r="R2" s="81" t="s">
+      <c r="P2" s="88"/>
+      <c r="Q2" s="89"/>
+      <c r="R2" s="87" t="s">
         <v>152</v>
       </c>
-      <c r="S2" s="82"/>
-      <c r="T2" s="82"/>
-      <c r="U2" s="82"/>
-      <c r="V2" s="83"/>
-      <c r="W2" s="81" t="s">
+      <c r="S2" s="88"/>
+      <c r="T2" s="88"/>
+      <c r="U2" s="88"/>
+      <c r="V2" s="89"/>
+      <c r="W2" s="87" t="s">
         <v>163</v>
       </c>
-      <c r="X2" s="82"/>
-      <c r="Y2" s="83"/>
-      <c r="Z2" s="81" t="s">
+      <c r="X2" s="88"/>
+      <c r="Y2" s="89"/>
+      <c r="Z2" s="87" t="s">
         <v>170</v>
       </c>
-      <c r="AA2" s="82"/>
-      <c r="AB2" s="82"/>
-      <c r="AC2" s="82"/>
-      <c r="AD2" s="82"/>
-      <c r="AE2" s="82"/>
-      <c r="AF2" s="82"/>
-      <c r="AG2" s="82"/>
-      <c r="AH2" s="82"/>
-      <c r="AI2" s="83"/>
-      <c r="AJ2" s="81" t="s">
+      <c r="AA2" s="88"/>
+      <c r="AB2" s="88"/>
+      <c r="AC2" s="88"/>
+      <c r="AD2" s="88"/>
+      <c r="AE2" s="88"/>
+      <c r="AF2" s="88"/>
+      <c r="AG2" s="88"/>
+      <c r="AH2" s="88"/>
+      <c r="AI2" s="89"/>
+      <c r="AJ2" s="87" t="s">
         <v>191</v>
       </c>
-      <c r="AK2" s="82"/>
-      <c r="AL2" s="82"/>
-      <c r="AM2" s="82"/>
-      <c r="AN2" s="82"/>
-      <c r="AO2" s="82"/>
-      <c r="AP2" s="82"/>
-      <c r="AQ2" s="82"/>
-      <c r="AR2" s="82"/>
-      <c r="AS2" s="83"/>
+      <c r="AK2" s="88"/>
+      <c r="AL2" s="88"/>
+      <c r="AM2" s="88"/>
+      <c r="AN2" s="88"/>
+      <c r="AO2" s="88"/>
+      <c r="AP2" s="88"/>
+      <c r="AQ2" s="88"/>
+      <c r="AR2" s="88"/>
+      <c r="AS2" s="89"/>
     </row>
     <row r="3" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A3" s="51" t="s">
@@ -11152,11 +11152,11 @@
       <c r="B3" s="52" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="80"/>
+      <c r="C3" s="86"/>
       <c r="D3" s="53" t="s">
         <v>124</v>
       </c>
-      <c r="E3" s="80"/>
+      <c r="E3" s="86"/>
       <c r="F3" s="53" t="s">
         <v>128</v>
       </c>
@@ -11344,6 +11344,9 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="F2:K2"/>
+    <mergeCell ref="L2:N2"/>
     <mergeCell ref="Z2:AI2"/>
     <mergeCell ref="AJ2:AS2"/>
     <mergeCell ref="W2:Y2"/>
@@ -11351,9 +11354,6 @@
     <mergeCell ref="C1:C3"/>
     <mergeCell ref="R2:V2"/>
     <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="F2:K2"/>
-    <mergeCell ref="L2:N2"/>
   </mergeCells>
   <dataValidations count="6">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Metadata and VCF" prompt="These sample names must match those provided in the VCF file(s)" sqref="B4:B1003 E1" xr:uid="{00000000-0002-0000-0700-000000000000}">

</xml_diff>